<commit_message>
avancée merge sur le siret
</commit_message>
<xml_diff>
--- a/Fichier ICPE_composants.xlsx
+++ b/Fichier ICPE_composants.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esthe\OneDrive\Documents\Mines\Semestre_2\Hackaton_entreprises_emettrices\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC9C94F6-E07E-4344-B958-79B827929BF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAAC52B3-B244-4C5C-80AE-B77A554B485F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FE0F0669-BFFF-48BA-AF26-0BA071A0680F}"/>
   </bookViews>
@@ -36,6 +36,32 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+  <si>
+    <t>Rubrique ICPE</t>
+  </si>
+  <si>
+    <t>Composants</t>
+  </si>
+  <si>
+    <t>NaN</t>
+  </si>
+  <si>
+    <t>Solide inflammable</t>
+  </si>
+  <si>
+    <t>Produits combustibles entrepot ouvert</t>
+  </si>
+  <si>
+    <t>Potasse caustique</t>
+  </si>
+  <si>
+    <t>Déchets non dangeureux non inertes</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -405,9 +431,84 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96F4EC86-0B83-4E38-BE87-2EE2E8DAF75E}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2980</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1450</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1510</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1630</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2718</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>4801</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>2510</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>3532</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>